<commit_message>
New refactored code for Drpodown
</commit_message>
<xml_diff>
--- a/src/test/resources/DataSet.xlsx
+++ b/src/test/resources/DataSet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\eclipse-workspace\PreVista\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50588A6A-F160-4167-85BD-04BA2D3C0DF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35070EAD-C435-433D-A4C9-8ECE49AC7FE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
     <t>Password</t>
   </si>
   <si>
-    <t>Vivek123456</t>
+    <t>Vivek1234567</t>
   </si>
 </sst>
 </file>

</xml_diff>